<commit_message>
docs: resync data dictionary with migrations 0009/0010
Renomme llm_provider -> llm_model (VARCHAR(20)->(64)), ajoute
prompt_version/created_at/updated_at (0009) et reviewed_at/review_status/
review_note (0010) sur la table regle. Nouvelle catégorie « Revue
manuelle » dans la feuille Légende : ces trois derniers champs sont saisis
à la main (psql), pas générés par le pipeline — contrairement à ce que
suggérait leur ancien rattachement implicite à « Généré par IA ».

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/conception/2_ingestion/A_dictionnaire_donnees_qualicheck.xlsx
+++ b/conception/2_ingestion/A_dictionnaire_donnees_qualicheck.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champs" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contraintes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remarques techniques" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Légende" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Champs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Contraintes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Remarques techniques" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Légende" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -55,7 +55,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -97,6 +97,12 @@
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E1D5E7"/>
+        <bgColor rgb="00E1D5E7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -124,7 +130,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -183,6 +189,8 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -548,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1094,12 +1102,12 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>llm_provider</t>
+          <t>llm_model</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>VARCHAR(20)</t>
+          <t>VARCHAR(64)</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -1109,643 +1117,643 @@
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Modèle LLM utilisé à l'ingestion — benchmark</t>
+          <t>Nom logique du modèle LLM — résolu via manifest.yml, jamais un nom de déploiement Azure codé en dur</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>gpt54_nano, kimi, mistral_small</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr"/>
-      <c r="H15" s="7" t="inlineStr"/>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Renommé depuis llm_provider, élargi VARCHAR(20)→(64) (migration 0009)</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>regle</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>prompt_version</t>
+        </is>
+      </c>
+      <c r="C16" s="20" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="D16" s="20" t="inlineStr">
+        <is>
+          <t>Généré par IA</t>
+        </is>
+      </c>
+      <c r="E16" s="20" t="inlineStr">
+        <is>
+          <t>Version du prompt d'enrichissement utilisée (frontmatter enrich_rule.md)</t>
+        </is>
+      </c>
+      <c r="F16" s="20" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
+      <c r="G16" s="20" t="n"/>
+      <c r="H16" s="20" t="inlineStr">
+        <is>
+          <t>NULL = produit avant l'instrumentation (migration 0009)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="20" t="inlineStr">
+        <is>
+          <t>regle</t>
+        </is>
+      </c>
+      <c r="B17" s="20" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="C17" s="20" t="inlineStr">
+        <is>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="D17" s="20" t="inlineStr">
+        <is>
+          <t>Généré par IA</t>
+        </is>
+      </c>
+      <c r="E17" s="20" t="inlineStr">
+        <is>
+          <t>Date de première création de la ligne (ingestion initiale)</t>
+        </is>
+      </c>
+      <c r="F17" s="20" t="n"/>
+      <c r="G17" s="20" t="n"/>
+      <c r="H17" s="20" t="inlineStr">
+        <is>
+          <t>NULL = produit avant l'instrumentation (migration 0009). Posé une seule fois, jamais réécrit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="20" t="inlineStr">
+        <is>
+          <t>regle</t>
+        </is>
+      </c>
+      <c r="B18" s="20" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="inlineStr">
+        <is>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="D18" s="20" t="inlineStr">
+        <is>
+          <t>Généré par IA</t>
+        </is>
+      </c>
+      <c r="E18" s="20" t="inlineStr">
+        <is>
+          <t>Date de dernière mise à jour de la ligne (ré-ingestion)</t>
+        </is>
+      </c>
+      <c r="F18" s="20" t="n"/>
+      <c r="G18" s="20" t="n"/>
+      <c r="H18" s="20" t="inlineStr">
+        <is>
+          <t>NULL = produit avant l'instrumentation (migration 0009). Mis à jour à chaque ré-ingestion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t>regle</t>
+        </is>
+      </c>
+      <c r="B19" s="21" t="inlineStr">
+        <is>
+          <t>reviewed_at</t>
+        </is>
+      </c>
+      <c r="C19" s="21" t="inlineStr">
+        <is>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="D19" s="21" t="inlineStr">
+        <is>
+          <t>Revue manuelle</t>
+        </is>
+      </c>
+      <c r="E19" s="21" t="inlineStr">
+        <is>
+          <t>Date de la dernière revue manuelle du classement produit par le LLM</t>
+        </is>
+      </c>
+      <c r="F19" s="21" t="n"/>
+      <c r="G19" s="21" t="n"/>
+      <c r="H19" s="21" t="inlineStr">
+        <is>
+          <t>NULL = pas encore revue manuellement. Jamais touché par le pipeline d'ingestion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>regle</t>
+        </is>
+      </c>
+      <c r="B20" s="21" t="inlineStr">
+        <is>
+          <t>review_status</t>
+        </is>
+      </c>
+      <c r="C20" s="21" t="inlineStr">
+        <is>
+          <t>VARCHAR(16)</t>
+        </is>
+      </c>
+      <c r="D20" s="21" t="inlineStr">
+        <is>
+          <t>Revue manuelle</t>
+        </is>
+      </c>
+      <c r="E20" s="21" t="inlineStr">
+        <is>
+          <t>Statut de la revue manuelle du classement</t>
+        </is>
+      </c>
+      <c r="F20" s="21" t="inlineStr">
+        <is>
+          <t>valide, a_revoir, invalide</t>
+        </is>
+      </c>
+      <c r="G20" s="21" t="n"/>
+      <c r="H20" s="21" t="inlineStr">
+        <is>
+          <t>Saisi manuellement (psql), pas de script dédié à ce stade</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t>regle</t>
+        </is>
+      </c>
+      <c r="B21" s="21" t="inlineStr">
+        <is>
+          <t>review_note</t>
+        </is>
+      </c>
+      <c r="C21" s="21" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D21" s="21" t="inlineStr">
+        <is>
+          <t>Revue manuelle</t>
+        </is>
+      </c>
+      <c r="E21" s="21" t="inlineStr">
+        <is>
+          <t>Notes libres du relecteur — matière pour un futur script de réécriture ciblée (enrich_again)</t>
+        </is>
+      </c>
+      <c r="F21" s="21" t="n"/>
+      <c r="G21" s="21" t="n"/>
+      <c r="H21" s="21" t="inlineStr">
+        <is>
+          <t>Saisi manuellement (psql)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>regle</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>embedding</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>vector(384)</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>Généré par IA</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E22" s="7" t="inlineStr">
         <is>
           <t>Vecteur pgvector — All MiniLM L12 v2</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F22" s="7" t="inlineStr">
         <is>
           <t>384 dimensions</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr"/>
-      <c r="H16" s="7" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr"/>
+      <c r="H22" s="7" t="inlineStr">
         <is>
           <t>Index HNSW sur cette colonne</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>objectif</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>COUNTER</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>Référentiel Opquast</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>Identifiant unique</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t>Auto-incrémenté</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>PK, NOT NULL</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr"/>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="H23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>objectif</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>objectif</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>VARCHAR(256)</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>Référentiel Opquast</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>Description de l'objectif qualité</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="F24" s="5" t="inlineStr">
         <is>
           <t>Améliorer l'accessibilité des contenus</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="G24" s="4" t="inlineStr">
         <is>
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="H18" s="5" t="inlineStr"/>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="H24" s="5" t="inlineStr"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>phase</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>COUNTER</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>Référentiel Opquast</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>Identifiant unique</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="F25" s="5" t="inlineStr">
         <is>
           <t>Auto-incrémenté</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>PK, NOT NULL</t>
         </is>
       </c>
-      <c r="H19" s="5" t="inlineStr"/>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="H25" s="5" t="inlineStr"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>phase</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>phase</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>VARCHAR(64)</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>Référentiel Opquast</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>Nom de la phase projet</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>Conception, Développement, Editorial, Recette</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr">
         <is>
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="H20" s="5" t="inlineStr"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="H26" s="5" t="inlineStr"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>tag</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>COUNTER</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>Référentiel Opquast</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t>Identifiant unique</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F27" s="5" t="inlineStr">
         <is>
           <t>Auto-incrémenté</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="G27" s="4" t="inlineStr">
         <is>
           <t>PK, NOT NULL</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr"/>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="H27" s="5" t="inlineStr"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>tag</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>tag</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>VARCHAR(50)</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>Référentiel Opquast</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E28" s="5" t="inlineStr">
         <is>
           <t>Libellé du tag</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="F28" s="5" t="inlineStr">
         <is>
           <t>Accessibilité, SEO, Écoconception</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="G28" s="4" t="inlineStr">
         <is>
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="H22" s="5" t="inlineStr"/>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="H28" s="5" t="inlineStr"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>utilisateur</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
+      <c r="C29" s="9" t="inlineStr">
         <is>
           <t>COUNTER</t>
         </is>
       </c>
-      <c r="D23" s="9" t="inlineStr">
+      <c r="D29" s="9" t="inlineStr">
         <is>
           <t>Cœur métier</t>
         </is>
       </c>
-      <c r="E23" s="10" t="inlineStr">
+      <c r="E29" s="10" t="inlineStr">
         <is>
           <t>Identifiant unique</t>
         </is>
       </c>
-      <c r="F23" s="10" t="inlineStr">
+      <c r="F29" s="10" t="inlineStr">
         <is>
           <t>Auto-incrémenté</t>
         </is>
       </c>
-      <c r="G23" s="9" t="inlineStr">
+      <c r="G29" s="9" t="inlineStr">
         <is>
           <t>PK, NOT NULL</t>
         </is>
       </c>
-      <c r="H23" s="10" t="inlineStr">
+      <c r="H29" s="10" t="inlineStr">
         <is>
           <t>MVP : utilisateur simulé</t>
         </is>
       </c>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>utilisateur</t>
-        </is>
-      </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>nom</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(64)</t>
-        </is>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>Cœur métier</t>
-        </is>
-      </c>
-      <c r="E24" s="10" t="inlineStr">
-        <is>
-          <t>Nom de l'utilisateur</t>
-        </is>
-      </c>
-      <c r="F24" s="10" t="inlineStr"/>
-      <c r="G24" s="9" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="H24" s="10" t="inlineStr"/>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>utilisateur</t>
-        </is>
-      </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>prenom</t>
-        </is>
-      </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(64)</t>
-        </is>
-      </c>
-      <c r="D25" s="9" t="inlineStr">
-        <is>
-          <t>Cœur métier</t>
-        </is>
-      </c>
-      <c r="E25" s="10" t="inlineStr">
-        <is>
-          <t>Prénom de l'utilisateur</t>
-        </is>
-      </c>
-      <c r="F25" s="10" t="inlineStr"/>
-      <c r="G25" s="9" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="H25" s="10" t="inlineStr"/>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="8" t="inlineStr">
-        <is>
-          <t>audit</t>
-        </is>
-      </c>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>COUNTER</t>
-        </is>
-      </c>
-      <c r="D26" s="9" t="inlineStr">
-        <is>
-          <t>Cœur métier</t>
-        </is>
-      </c>
-      <c r="E26" s="10" t="inlineStr">
-        <is>
-          <t>Identifiant unique de l'audit</t>
-        </is>
-      </c>
-      <c r="F26" s="10" t="inlineStr">
-        <is>
-          <t>Auto-incrémenté</t>
-        </is>
-      </c>
-      <c r="G26" s="9" t="inlineStr">
-        <is>
-          <t>PK, NOT NULL</t>
-        </is>
-      </c>
-      <c r="H26" s="10" t="inlineStr"/>
-    </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="9" t="inlineStr">
-        <is>
-          <t>audit</t>
-        </is>
-      </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>url_depart</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(512)</t>
-        </is>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
-        <is>
-          <t>Cœur métier</t>
-        </is>
-      </c>
-      <c r="E27" s="10" t="inlineStr">
-        <is>
-          <t>URL racine du site audité</t>
-        </is>
-      </c>
-      <c r="F27" s="10" t="inlineStr">
-        <is>
-          <t>https://exemple.com</t>
-        </is>
-      </c>
-      <c r="G27" s="9" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="H27" s="10" t="inlineStr"/>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="9" t="inlineStr">
-        <is>
-          <t>audit</t>
-        </is>
-      </c>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>statut</t>
-        </is>
-      </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(50)</t>
-        </is>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
-        <is>
-          <t>Cœur métier</t>
-        </is>
-      </c>
-      <c r="E28" s="10" t="inlineStr">
-        <is>
-          <t>État de l'audit</t>
-        </is>
-      </c>
-      <c r="F28" s="10" t="inlineStr">
-        <is>
-          <t>en_cours, pret_dialogue, termine</t>
-        </is>
-      </c>
-      <c r="G28" s="9" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="H28" s="10" t="inlineStr"/>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>audit</t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>date_creation</t>
-        </is>
-      </c>
-      <c r="C29" s="9" t="inlineStr">
-        <is>
-          <t>DATETIME</t>
-        </is>
-      </c>
-      <c r="D29" s="9" t="inlineStr">
-        <is>
-          <t>Cœur métier</t>
-        </is>
-      </c>
-      <c r="E29" s="10" t="inlineStr">
-        <is>
-          <t>Date de création de l'audit</t>
-        </is>
-      </c>
-      <c r="F29" s="10" t="inlineStr"/>
-      <c r="G29" s="9" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="H29" s="10" t="inlineStr"/>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="9" t="inlineStr">
         <is>
+          <t>utilisateur</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>nom</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(64)</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>Cœur métier</t>
+        </is>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>Nom de l'utilisateur</t>
+        </is>
+      </c>
+      <c r="F30" s="10" t="inlineStr"/>
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="H30" s="10" t="inlineStr"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>utilisateur</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>prenom</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(64)</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>Cœur métier</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>Prénom de l'utilisateur</t>
+        </is>
+      </c>
+      <c r="F31" s="10" t="inlineStr"/>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="H31" s="10" t="inlineStr"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
           <t>audit</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>date_modification</t>
-        </is>
-      </c>
-      <c r="C30" s="9" t="inlineStr">
-        <is>
-          <t>DATETIME</t>
-        </is>
-      </c>
-      <c r="D30" s="9" t="inlineStr">
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>COUNTER</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
         <is>
           <t>Cœur métier</t>
         </is>
       </c>
-      <c r="E30" s="10" t="inlineStr">
-        <is>
-          <t>Date de dernière modification</t>
-        </is>
-      </c>
-      <c r="F30" s="10" t="inlineStr"/>
-      <c r="G30" s="9" t="inlineStr"/>
-      <c r="H30" s="10" t="inlineStr"/>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t>page</t>
-        </is>
-      </c>
-      <c r="B31" s="9" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="C31" s="9" t="inlineStr">
-        <is>
-          <t>COUNTER</t>
-        </is>
-      </c>
-      <c r="D31" s="9" t="inlineStr">
-        <is>
-          <t>Cœur métier</t>
-        </is>
-      </c>
-      <c r="E31" s="10" t="inlineStr">
-        <is>
-          <t>Identifiant unique de la page</t>
-        </is>
-      </c>
-      <c r="F31" s="10" t="inlineStr">
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>Identifiant unique de l'audit</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="inlineStr">
         <is>
           <t>Auto-incrémenté</t>
         </is>
       </c>
-      <c r="G31" s="9" t="inlineStr">
+      <c r="G32" s="9" t="inlineStr">
         <is>
           <t>PK, NOT NULL</t>
-        </is>
-      </c>
-      <c r="H31" s="10" t="inlineStr"/>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="9" t="inlineStr">
-        <is>
-          <t>page</t>
-        </is>
-      </c>
-      <c r="B32" s="9" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="C32" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(512)</t>
-        </is>
-      </c>
-      <c r="D32" s="9" t="inlineStr">
-        <is>
-          <t>Cœur métier</t>
-        </is>
-      </c>
-      <c r="E32" s="10" t="inlineStr">
-        <is>
-          <t>URL complète de la page</t>
-        </is>
-      </c>
-      <c r="F32" s="10" t="inlineStr">
-        <is>
-          <t>https://exemple.com/contact</t>
-        </is>
-      </c>
-      <c r="G32" s="9" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
         </is>
       </c>
       <c r="H32" s="10" t="inlineStr"/>
@@ -1753,17 +1761,17 @@
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>page</t>
+          <t>audit</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>titre</t>
+          <t>url_depart</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(255)</t>
+          <t>VARCHAR(512)</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
@@ -1773,31 +1781,35 @@
       </c>
       <c r="E33" s="10" t="inlineStr">
         <is>
-          <t>Titre HTML de la page</t>
+          <t>URL racine du site audité</t>
         </is>
       </c>
       <c r="F33" s="10" t="inlineStr">
         <is>
-          <t>Page de contact — Exemple</t>
-        </is>
-      </c>
-      <c r="G33" s="9" t="inlineStr"/>
+          <t>https://exemple.com</t>
+        </is>
+      </c>
+      <c r="G33" s="9" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
       <c r="H33" s="10" t="inlineStr"/>
     </row>
     <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="8" t="inlineStr">
-        <is>
-          <t>audit_page</t>
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>audit</t>
         </is>
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>statut_http</t>
+          <t>statut</t>
         </is>
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(10)</t>
+          <t>VARCHAR(50)</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
@@ -1807,35 +1819,35 @@
       </c>
       <c r="E34" s="10" t="inlineStr">
         <is>
-          <t>Code HTTP retourné lors du crawl</t>
+          <t>État de l'audit</t>
         </is>
       </c>
       <c r="F34" s="10" t="inlineStr">
         <is>
-          <t>200, 301, 404, 500</t>
-        </is>
-      </c>
-      <c r="G34" s="9" t="inlineStr"/>
-      <c r="H34" s="10" t="inlineStr">
-        <is>
-          <t>Stocké comme texte, sans calcul</t>
-        </is>
-      </c>
+          <t>en_cours, pret_dialogue, termine</t>
+        </is>
+      </c>
+      <c r="G34" s="9" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="H34" s="10" t="inlineStr"/>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>audit_page</t>
+          <t>audit</t>
         </is>
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>est_selectionnee</t>
+          <t>date_creation</t>
         </is>
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>LOGICAL</t>
+          <t>DATETIME</t>
         </is>
       </c>
       <c r="D35" s="9" t="inlineStr">
@@ -1845,14 +1857,10 @@
       </c>
       <c r="E35" s="10" t="inlineStr">
         <is>
-          <t>Page sélectionnée par l'auditeur pour cet audit</t>
-        </is>
-      </c>
-      <c r="F35" s="10" t="inlineStr">
-        <is>
-          <t>true, false</t>
-        </is>
-      </c>
+          <t>Date de création de l'audit</t>
+        </is>
+      </c>
+      <c r="F35" s="10" t="inlineStr"/>
       <c r="G35" s="9" t="inlineStr">
         <is>
           <t>NOT NULL</t>
@@ -1863,12 +1871,12 @@
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>audit_page</t>
+          <t>audit</t>
         </is>
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>date_crawl</t>
+          <t>date_modification</t>
         </is>
       </c>
       <c r="C36" s="9" t="inlineStr">
@@ -1883,7 +1891,7 @@
       </c>
       <c r="E36" s="10" t="inlineStr">
         <is>
-          <t>Date du crawl de la page</t>
+          <t>Date de dernière modification</t>
         </is>
       </c>
       <c r="F36" s="10" t="inlineStr"/>
@@ -1893,17 +1901,17 @@
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>constat</t>
+          <t>page</t>
         </is>
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>statut</t>
+          <t>id</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(32)</t>
+          <t>COUNTER</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
@@ -1913,17 +1921,17 @@
       </c>
       <c r="E37" s="10" t="inlineStr">
         <is>
-          <t>Résultat de l'analyse de la règle sur la page</t>
+          <t>Identifiant unique de la page</t>
         </is>
       </c>
       <c r="F37" s="10" t="inlineStr">
         <is>
-          <t>conforme, non_conforme, non_applicable</t>
+          <t>Auto-incrémenté</t>
         </is>
       </c>
       <c r="G37" s="9" t="inlineStr">
         <is>
-          <t>NOT NULL</t>
+          <t>PK, NOT NULL</t>
         </is>
       </c>
       <c r="H37" s="10" t="inlineStr"/>
@@ -1931,12 +1939,12 @@
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>constat</t>
+          <t>page</t>
         </is>
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>commentaire</t>
+          <t>url</t>
         </is>
       </c>
       <c r="C38" s="9" t="inlineStr">
@@ -1951,27 +1959,35 @@
       </c>
       <c r="E38" s="10" t="inlineStr">
         <is>
-          <t>Commentaire de l'agent sur le constat</t>
-        </is>
-      </c>
-      <c r="F38" s="10" t="inlineStr"/>
-      <c r="G38" s="9" t="inlineStr"/>
+          <t>URL complète de la page</t>
+        </is>
+      </c>
+      <c r="F38" s="10" t="inlineStr">
+        <is>
+          <t>https://exemple.com/contact</t>
+        </is>
+      </c>
+      <c r="G38" s="9" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
       <c r="H38" s="10" t="inlineStr"/>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>constat</t>
+          <t>page</t>
         </is>
       </c>
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>recommandation</t>
+          <t>titre</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(512)</t>
+          <t>VARCHAR(255)</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
@@ -1981,27 +1997,31 @@
       </c>
       <c r="E39" s="10" t="inlineStr">
         <is>
-          <t>Recommandation de correction proposée</t>
-        </is>
-      </c>
-      <c r="F39" s="10" t="inlineStr"/>
+          <t>Titre HTML de la page</t>
+        </is>
+      </c>
+      <c r="F39" s="10" t="inlineStr">
+        <is>
+          <t>Page de contact — Exemple</t>
+        </is>
+      </c>
       <c r="G39" s="9" t="inlineStr"/>
       <c r="H39" s="10" t="inlineStr"/>
     </row>
     <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="9" t="inlineStr">
-        <is>
-          <t>constat</t>
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>audit_page</t>
         </is>
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>preuve</t>
+          <t>statut_http</t>
         </is>
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(512)</t>
+          <t>VARCHAR(10)</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
@@ -2011,22 +2031,30 @@
       </c>
       <c r="E40" s="10" t="inlineStr">
         <is>
-          <t>Extrait HTML ou capture servant de preuve</t>
-        </is>
-      </c>
-      <c r="F40" s="10" t="inlineStr"/>
+          <t>Code HTTP retourné lors du crawl</t>
+        </is>
+      </c>
+      <c r="F40" s="10" t="inlineStr">
+        <is>
+          <t>200, 301, 404, 500</t>
+        </is>
+      </c>
       <c r="G40" s="9" t="inlineStr"/>
-      <c r="H40" s="10" t="inlineStr"/>
+      <c r="H40" s="10" t="inlineStr">
+        <is>
+          <t>Stocké comme texte, sans calcul</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>constat</t>
+          <t>audit_page</t>
         </is>
       </c>
       <c r="B41" s="9" t="inlineStr">
         <is>
-          <t>validation_humaine</t>
+          <t>est_selectionnee</t>
         </is>
       </c>
       <c r="C41" s="9" t="inlineStr">
@@ -2041,194 +2069,390 @@
       </c>
       <c r="E41" s="10" t="inlineStr">
         <is>
-          <t>Décision finale de l'auditeur</t>
+          <t>Page sélectionnée par l'auditeur pour cet audit</t>
         </is>
       </c>
       <c r="F41" s="10" t="inlineStr">
         <is>
-          <t>true (validé), false (rejeté), null (non traité)</t>
-        </is>
-      </c>
-      <c r="G41" s="9" t="inlineStr"/>
-      <c r="H41" s="10" t="inlineStr">
-        <is>
-          <t>Alimente strategie_score</t>
-        </is>
-      </c>
+          <t>true, false</t>
+        </is>
+      </c>
+      <c r="G41" s="9" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="H41" s="10" t="inlineStr"/>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="9" t="inlineStr">
         <is>
+          <t>audit_page</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>date_crawl</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>DATETIME</t>
+        </is>
+      </c>
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>Cœur métier</t>
+        </is>
+      </c>
+      <c r="E42" s="10" t="inlineStr">
+        <is>
+          <t>Date du crawl de la page</t>
+        </is>
+      </c>
+      <c r="F42" s="10" t="inlineStr"/>
+      <c r="G42" s="9" t="inlineStr"/>
+      <c r="H42" s="10" t="inlineStr"/>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
           <t>constat</t>
         </is>
       </c>
-      <c r="B42" s="9" t="inlineStr">
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>statut</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(32)</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>Cœur métier</t>
+        </is>
+      </c>
+      <c r="E43" s="10" t="inlineStr">
+        <is>
+          <t>Résultat de l'analyse de la règle sur la page</t>
+        </is>
+      </c>
+      <c r="F43" s="10" t="inlineStr">
+        <is>
+          <t>conforme, non_conforme, non_applicable</t>
+        </is>
+      </c>
+      <c r="G43" s="9" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="H43" s="10" t="inlineStr"/>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
+          <t>constat</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>commentaire</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(512)</t>
+        </is>
+      </c>
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>Cœur métier</t>
+        </is>
+      </c>
+      <c r="E44" s="10" t="inlineStr">
+        <is>
+          <t>Commentaire de l'agent sur le constat</t>
+        </is>
+      </c>
+      <c r="F44" s="10" t="inlineStr"/>
+      <c r="G44" s="9" t="inlineStr"/>
+      <c r="H44" s="10" t="inlineStr"/>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>constat</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>recommandation</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(512)</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>Cœur métier</t>
+        </is>
+      </c>
+      <c r="E45" s="10" t="inlineStr">
+        <is>
+          <t>Recommandation de correction proposée</t>
+        </is>
+      </c>
+      <c r="F45" s="10" t="inlineStr"/>
+      <c r="G45" s="9" t="inlineStr"/>
+      <c r="H45" s="10" t="inlineStr"/>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>constat</t>
+        </is>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>preuve</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(512)</t>
+        </is>
+      </c>
+      <c r="D46" s="9" t="inlineStr">
+        <is>
+          <t>Cœur métier</t>
+        </is>
+      </c>
+      <c r="E46" s="10" t="inlineStr">
+        <is>
+          <t>Extrait HTML ou capture servant de preuve</t>
+        </is>
+      </c>
+      <c r="F46" s="10" t="inlineStr"/>
+      <c r="G46" s="9" t="inlineStr"/>
+      <c r="H46" s="10" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="9" t="inlineStr">
+        <is>
+          <t>constat</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>validation_humaine</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>LOGICAL</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>Cœur métier</t>
+        </is>
+      </c>
+      <c r="E47" s="10" t="inlineStr">
+        <is>
+          <t>Décision finale de l'auditeur</t>
+        </is>
+      </c>
+      <c r="F47" s="10" t="inlineStr">
+        <is>
+          <t>true (validé), false (rejeté), null (non traité)</t>
+        </is>
+      </c>
+      <c r="G47" s="9" t="inlineStr"/>
+      <c r="H47" s="10" t="inlineStr">
+        <is>
+          <t>Alimente strategie_score</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>constat</t>
+        </is>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
         <is>
           <t>feedback_auditeur</t>
         </is>
       </c>
-      <c r="C42" s="9" t="inlineStr">
+      <c r="C48" s="9" t="inlineStr">
         <is>
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D42" s="9" t="inlineStr">
+      <c r="D48" s="9" t="inlineStr">
         <is>
           <t>Cœur métier</t>
         </is>
       </c>
-      <c r="E42" s="10" t="inlineStr">
+      <c r="E48" s="10" t="inlineStr">
         <is>
           <t>Commentaire qualitatif de l'auditeur sur le constat</t>
         </is>
       </c>
-      <c r="F42" s="10" t="inlineStr">
+      <c r="F48" s="10" t="inlineStr">
         <is>
           <t>Constat trop générique, Playwright inutile ici</t>
         </is>
       </c>
-      <c r="G42" s="9" t="inlineStr"/>
-      <c r="H42" s="10" t="inlineStr">
+      <c r="G48" s="9" t="inlineStr"/>
+      <c r="H48" s="10" t="inlineStr">
         <is>
           <t>Base de la feedback loop post-MVP</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="11" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="11" t="inlineStr">
         <is>
           <t>objectif_regle</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
+      <c r="B49" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C43" s="12" t="inlineStr">
+      <c r="C49" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D43" s="12" t="inlineStr">
+      <c r="D49" s="12" t="inlineStr">
         <is>
           <t>Association</t>
         </is>
       </c>
-      <c r="E43" s="13" t="inlineStr">
+      <c r="E49" s="13" t="inlineStr">
         <is>
           <t>Lien many-to-many entre objectif et regle</t>
         </is>
       </c>
-      <c r="F43" s="13" t="inlineStr"/>
-      <c r="G43" s="12" t="inlineStr">
+      <c r="F49" s="13" t="inlineStr"/>
+      <c r="G49" s="12" t="inlineStr">
         <is>
           <t>FK objectif.id, FK regle.id</t>
         </is>
       </c>
-      <c r="H43" s="13" t="inlineStr"/>
-    </row>
-    <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="11" t="inlineStr">
+      <c r="H49" s="13" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="11" t="inlineStr">
         <is>
           <t>phase_regle</t>
         </is>
       </c>
-      <c r="B44" s="12" t="inlineStr">
+      <c r="B50" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C44" s="12" t="inlineStr">
+      <c r="C50" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D44" s="12" t="inlineStr">
+      <c r="D50" s="12" t="inlineStr">
         <is>
           <t>Association</t>
         </is>
       </c>
-      <c r="E44" s="13" t="inlineStr">
+      <c r="E50" s="13" t="inlineStr">
         <is>
           <t>Lien many-to-many entre phase et regle</t>
         </is>
       </c>
-      <c r="F44" s="13" t="inlineStr"/>
-      <c r="G44" s="12" t="inlineStr">
+      <c r="F50" s="13" t="inlineStr"/>
+      <c r="G50" s="12" t="inlineStr">
         <is>
           <t>FK phase.id, FK regle.id</t>
         </is>
       </c>
-      <c r="H44" s="13" t="inlineStr"/>
-    </row>
-    <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="11" t="inlineStr">
+      <c r="H50" s="13" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="inlineStr">
         <is>
           <t>regle_tag</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
+      <c r="B51" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C45" s="12" t="inlineStr">
+      <c r="C51" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D45" s="12" t="inlineStr">
+      <c r="D51" s="12" t="inlineStr">
         <is>
           <t>Association</t>
         </is>
       </c>
-      <c r="E45" s="13" t="inlineStr">
+      <c r="E51" s="13" t="inlineStr">
         <is>
           <t>Lien many-to-many entre regle et tag</t>
         </is>
       </c>
-      <c r="F45" s="13" t="inlineStr"/>
-      <c r="G45" s="12" t="inlineStr">
+      <c r="F51" s="13" t="inlineStr"/>
+      <c r="G51" s="12" t="inlineStr">
         <is>
           <t>FK regle.id, FK tag.id</t>
         </is>
       </c>
-      <c r="H45" s="13" t="inlineStr"/>
-    </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="11" t="inlineStr">
+      <c r="H51" s="13" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="11" t="inlineStr">
         <is>
           <t>audit_regle</t>
         </is>
       </c>
-      <c r="B46" s="12" t="inlineStr">
+      <c r="B52" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C46" s="12" t="inlineStr">
+      <c r="C52" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D46" s="12" t="inlineStr">
+      <c r="D52" s="12" t="inlineStr">
         <is>
           <t>Association</t>
         </is>
       </c>
-      <c r="E46" s="13" t="inlineStr">
+      <c r="E52" s="13" t="inlineStr">
         <is>
           <t>Règles sélectionnées pour un audit</t>
         </is>
       </c>
-      <c r="F46" s="13" t="inlineStr"/>
-      <c r="G46" s="12" t="inlineStr">
+      <c r="F52" s="13" t="inlineStr"/>
+      <c r="G52" s="12" t="inlineStr">
         <is>
           <t>FK audit.id, FK regle.id</t>
         </is>
       </c>
-      <c r="H46" s="13" t="inlineStr"/>
+      <c r="H52" s="13" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2900,7 +3124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2962,6 +3186,18 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>Revue manuelle</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Champs saisis manuellement par un relecteur humain (psql), jamais par le pipeline d'ingestion.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>

</xml_diff>